<commit_message>
Enable pytest for testing framework; refactor test executor and keyword engine for improved functionality and compatibility
</commit_message>
<xml_diff>
--- a/framework/data/excel/login_hybrid.xlsx
+++ b/framework/data/excel/login_hybrid.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\_DA\DA4\framework\data\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DA4\DA4_hybrid_selenium_framework\framework\data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4E0BEA-9D7C-425B-8F1C-64265F22E66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAC07EE6-A8AA-4D4A-8319-CD8A36D7B73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2415" yWindow="4140" windowWidth="12450" windowHeight="13185" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test_steps" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="59">
   <si>
     <t>template_id</t>
   </si>
@@ -197,19 +197,7 @@
     <t>LOGIN_07</t>
   </si>
   <si>
-    <t xml:space="preserve"> validUser </t>
-  </si>
-  <si>
-    <t>Kiem tra username co khoang trang dau/cuoi. Can xac nhan demoqa co trim du lieu truoc khi hien thi hay khong truoc khi chay that.</t>
-  </si>
-  <si>
-    <t>LOGIN_08</t>
-  </si>
-  <si>
     <t>AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
-  </si>
-  <si>
-    <t>Gia tri 500 ky tu la du lieu bien; expected_maxlength dang de trong - can kiem tra thuoc tinh maxlength thuc te tren o username cua demoqa truoc khi dien va chay.</t>
   </si>
 </sst>
 </file>
@@ -619,10 +607,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
@@ -630,7 +618,7 @@
     <col min="6" max="6" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -650,7 +638,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -666,7 +654,7 @@
       </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -684,7 +672,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -702,7 +690,7 @@
       </c>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -718,7 +706,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -734,7 +722,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -752,7 +740,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -768,7 +756,7 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>21</v>
       </c>
@@ -786,7 +774,7 @@
       </c>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -804,7 +792,7 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>21</v>
       </c>
@@ -820,7 +808,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
@@ -838,7 +826,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>24</v>
       </c>
@@ -854,7 +842,7 @@
       </c>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -872,7 +860,7 @@
       </c>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>24</v>
       </c>
@@ -890,7 +878,7 @@
       </c>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>24</v>
       </c>
@@ -906,7 +894,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>24</v>
       </c>
@@ -924,7 +912,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>24</v>
       </c>
@@ -942,7 +930,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>28</v>
       </c>
@@ -958,7 +946,7 @@
       </c>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>28</v>
       </c>
@@ -976,38 +964,73 @@
       </c>
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="4">
         <v>3</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="4">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="2">
+        <v>5</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>31</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="34.5703125" customWidth="1"/>
+    <col min="2" max="2" width="34.5546875" customWidth="1"/>
     <col min="3" max="3" width="45" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -1018,7 +1041,7 @@
     <col min="11" max="11" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -1053,7 +1076,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>42</v>
       </c>
@@ -1078,7 +1101,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>46</v>
       </c>
@@ -1101,7 +1124,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>49</v>
       </c>
@@ -1124,7 +1147,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>52</v>
       </c>
@@ -1145,7 +1168,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>54</v>
       </c>
@@ -1168,7 +1191,7 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>56</v>
       </c>
@@ -1191,12 +1214,12 @@
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>58</v>
@@ -1204,43 +1227,19 @@
       <c r="D8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="51" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="6" t="s">
-        <v>62</v>
-      </c>
+      <c r="J8" s="2">
+        <v>250</v>
+      </c>
+      <c r="K8" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: support multi-website testing and JavaScript Alert verification
</commit_message>
<xml_diff>
--- a/framework/data/excel/login_hybrid.xlsx
+++ b/framework/data/excel/login_hybrid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\_DA\DA4\framework\data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80AEF14E-14FC-42C7-A966-0F2BBCDC7E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D7F015-FC9D-431F-8BEE-6B9892271B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="3240" windowWidth="12450" windowHeight="13185" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="3810" windowWidth="12450" windowHeight="13185" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test_steps" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="89">
   <si>
     <t>template_id</t>
   </si>
@@ -80,12 +80,6 @@
     <t>verifyText</t>
   </si>
   <si>
-    <t>login.userNameLabel</t>
-  </si>
-  <si>
-    <t>{expected_username_label}</t>
-  </si>
-  <si>
     <t>LOGIN_INVALID_CREDENTIALS</t>
   </si>
   <si>
@@ -131,9 +125,6 @@
     <t>expected_url</t>
   </si>
   <si>
-    <t>expected_username_label</t>
-  </si>
-  <si>
     <t>expected_message</t>
   </si>
   <si>
@@ -201,13 +192,109 @@
   </si>
   <si>
     <t>&lt;empty&gt;</t>
+  </si>
+  <si>
+    <t>website</t>
+  </si>
+  <si>
+    <t>demoQA</t>
+  </si>
+  <si>
+    <t>taophoBA</t>
+  </si>
+  <si>
+    <t>ts</t>
+  </si>
+  <si>
+    <t>TS_LOGIN_INVALID_CREDENTIALS</t>
+  </si>
+  <si>
+    <t>Navigate</t>
+  </si>
+  <si>
+    <t>SetText</t>
+  </si>
+  <si>
+    <t>ClickElement</t>
+  </si>
+  <si>
+    <t>VerifyAlert</t>
+  </si>
+  <si>
+    <t>TS_LOGIN_MAX_LENGTH</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_01</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_02</t>
+  </si>
+  <si>
+    <t>Tên đăng nhập hoặc mật khẩu không đúng!</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_03</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_04</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_05</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_06</t>
+  </si>
+  <si>
+    <t>LOGIN_TS_07</t>
+  </si>
+  <si>
+    <t>Tên đăng nhập không được vượt quá 250 ký tự!</t>
+  </si>
+  <si>
+    <t>admin1</t>
+  </si>
+  <si>
+    <t>adadad</t>
+  </si>
+  <si>
+    <t>/admin/admin.html</t>
+  </si>
+  <si>
+    <t>admin@taopho.com</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_01</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_02</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_03</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_04</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_05</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_06</t>
+  </si>
+  <si>
+    <t>LOGIN_TPBA_07</t>
+  </si>
+  <si>
+    <t>Email/số điện thoại/tên tài khoản hoặc mật khẩu không đúng!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,8 +324,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -266,8 +381,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9EFF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9EFF7"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -290,11 +429,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -317,12 +472,48 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFE9EFF7"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -619,7 +810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
@@ -735,299 +926,449 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="4">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="2">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="4">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="2">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="4">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="2">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="4">
+        <v>3</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="2">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="4">
+        <v>5</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
-        <v>6</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="2">
+      <c r="C17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="9">
         <v>1</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C18" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2" t="s">
+      <c r="D18" s="9"/>
+      <c r="E18" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="4">
+      <c r="F18" s="10"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="11">
         <v>2</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C19" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D19" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E19" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="5"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="2">
-        <v>3</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="4">
-        <v>4</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="2">
-        <v>5</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="4">
-        <v>1</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="2">
-        <v>2</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="4">
-        <v>3</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="2">
-        <v>4</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="3"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="4">
-        <v>5</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="2">
-        <v>6</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="2">
-        <v>1</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="3"/>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B20" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="11">
+        <v>4</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="9">
+        <v>5</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="8">
+        <v>1</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="14">
+        <v>2</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="4">
+      <c r="F24" s="14"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="8">
         <v>3</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="C25" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E25" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="4">
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="14">
         <v>4</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="C26" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="5"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="2">
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="8">
         <v>5</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="C27" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" s="14">
+        <v>1</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" s="14"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" s="8">
+        <v>2</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>31</v>
+      <c r="E29" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" s="14">
+        <v>3</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="14"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="8">
+        <v>4</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B32" s="14">
+        <v>5</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1038,74 +1379,75 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="34.5703125" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="27" customWidth="1"/>
-    <col min="7" max="7" width="33" customWidth="1"/>
-    <col min="8" max="9" width="27" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="60.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -1114,22 +1456,24 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>46</v>
+      <c r="A3" t="s">
+        <v>58</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="4"/>
+        <v>40</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -1137,22 +1481,24 @@
       <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>49</v>
+      <c r="A4" t="s">
+        <v>58</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1160,94 +1506,102 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>52</v>
+      <c r="A5" t="s">
+        <v>58</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="4"/>
+        <v>56</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>54</v>
+      <c r="A6" t="s">
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>57</v>
+    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>58</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -1257,9 +1611,375 @@
       </c>
       <c r="K8" s="6"/>
     </row>
+    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="18"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="I19" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="18"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D16" r:id="rId1" xr:uid="{B361B021-C219-43F4-B5EB-E9F8D67BB841}"/>
+    <hyperlink ref="D17" r:id="rId2" xr:uid="{DB5F175B-9E5C-4E09-BEF6-79EF0E672F15}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>